<commit_message>
Refresh Epic Realty copy as plain paragraphs without dash lists.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/portfolio/epic-realty/Epic Realty.xlsx
+++ b/public/portfolio/epic-realty/Epic Realty.xlsx
@@ -20,10 +20,13 @@
     <t>Epic Realty</t>
   </si>
   <si>
+    <t>Wrzucasz do folderu projektu</t>
+  </si>
+  <si>
     <t>Sekcja</t>
   </si>
   <si>
-    <t>Wrzucasz do folderu projektu</t>
+    <t>Co robi</t>
   </si>
   <si>
     <t>Pole</t>
@@ -32,61 +35,70 @@
     <t>EN</t>
   </si>
   <si>
-    <t>Co robi</t>
-  </si>
-  <si>
     <t>PL</t>
   </si>
   <si>
+    <t>Jak używać</t>
+  </si>
+  <si>
     <t>ES</t>
   </si>
   <si>
     <t>Uwagi</t>
   </si>
   <si>
-    <t>Jak używać</t>
+    <t>1. Skopiuj plik i nazwij np. Epic Realty.xlsx (jeden Excel = jeden projekt).</t>
   </si>
   <si>
     <t>cover.webp / cover.webm / cover.mp4</t>
   </si>
   <si>
-    <t>1. Skopiuj plik i nazwij np. Epic Realty.xlsx (jeden Excel = jeden projekt).</t>
-  </si>
-  <si>
     <t>Okładka na liście projektów</t>
   </si>
   <si>
     <t>Start</t>
   </si>
   <si>
+    <t>2. W karcie „Projekt” uzupełnij EN, PL i ES — tylko teksty.</t>
+  </si>
+  <si>
     <t>slug</t>
   </si>
   <si>
     <t>epic-realty</t>
   </si>
   <si>
-    <t>2. W karcie „Projekt” uzupełnij EN, PL i ES — tylko teksty.</t>
-  </si>
-  <si>
     <t>bg.webp</t>
   </si>
   <si>
     <t>Tło hero na stronie projektu</t>
   </si>
   <si>
+    <t>3. Wrzuć grafiki do public/portfolio/{folderName}/ (cover, bg, 1.webp, 2.webp…).</t>
+  </si>
+  <si>
+    <t>4. Wyślij mi Excel albo wrzuć go do tego folderu — ja wciągam treści.</t>
+  </si>
+  <si>
+    <t>1.webp</t>
+  </si>
+  <si>
+    <t>Grafika przy Overview (opcjonalnie)</t>
+  </si>
+  <si>
     <t>Nazwa pliku projektu, np. epic-realty (→ epic-realty.md). Tylko EN.</t>
   </si>
   <si>
-    <t>3. Wrzuć grafiki do public/portfolio/{folderName}/ (cover, bg, 1.webp, 2.webp…).</t>
-  </si>
-  <si>
-    <t>1.webp</t>
-  </si>
-  <si>
-    <t>Grafika przy Overview (opcjonalnie)</t>
-  </si>
-  <si>
-    <t>4. Wyślij mi Excel albo wrzuć go do tego folderu — ja wciągam treści.</t>
+    <t>Co jest automatyczne (nie wpisujesz w Excelu)</t>
+  </si>
+  <si>
+    <t>2.webp, 3.webp, 4.webp…</t>
+  </si>
+  <si>
+    <t>Pełne kadry w galerii (kolejność = numer)</t>
+  </si>
+  <si>
+    <t>Zdjęcia i wideo: cover.webp/mp4, bg.webp, 1.webp (overview), 2.webp / 2.1+2.2… — strona czyta je z folderu. Nie ma pól afterGroup / ścieżek grafik.</t>
   </si>
   <si>
     <t>folderName</t>
@@ -95,51 +107,45 @@
     <t/>
   </si>
   <si>
-    <t>2.webp, 3.webp, 4.webp…</t>
-  </si>
-  <si>
-    <t>Pełne kadry w galerii (kolejność = numer)</t>
-  </si>
-  <si>
-    <t>Co jest automatyczne (nie wpisujesz w Excelu)</t>
+    <t>Układ i kolory sekcji: theme idzie automatycznie (dark → light → muted). Overview zawsze jasny. Sekcja Summary / Podsumowanie / Resultado zawsze na końcu.</t>
+  </si>
+  <si>
+    <t>2.1.webp + 2.2.webp…</t>
+  </si>
+  <si>
+    <t>Pary pod pełnym kadrem o tym samym numerze</t>
+  </si>
+  <si>
+    <t>CAPS (etykiety, tytuły, info) robi CSS na stronie — w Excelu pisz normalnie. Nawiasów [ ] przy labelach nie dopisuj.</t>
   </si>
   <si>
     <t>Folder grafik: public/portfolio/{folderName}/. Zdjęcia bierze strona sama. Tylko EN.</t>
   </si>
   <si>
+    <t>Pola tylko EN (żółte i tak wypełnij w kolumnie EN)</t>
+  </si>
+  <si>
     <t>order</t>
   </si>
   <si>
-    <t>2.1.webp + 2.2.webp…</t>
-  </si>
-  <si>
-    <t>Pary pod pełnym kadrem o tym samym numerze</t>
-  </si>
-  <si>
-    <t>Zdjęcia i wideo: cover.webp/mp4, bg.webp, 1.webp (overview), 2.webp / 2.1+2.2… — strona czyta je z folderu. Nie ma pól afterGroup / ścieżek grafik.</t>
+    <t>ten Excel (opcjonalnie)</t>
+  </si>
+  <si>
+    <t>Żebym mógł wciągnąć teksty z folderu</t>
+  </si>
+  <si>
+    <t>slug, folderName, order, comingSoon, categories, year, liveUrl.</t>
   </si>
   <si>
     <t>Kolejność na liście (1, 2, 3…). Mniejsza = wyżej. Tylko EN.</t>
   </si>
   <si>
-    <t>Układ i kolory sekcji: theme idzie automatycznie (dark → light → muted). Overview zawsze jasny. Sekcja Summary / Podsumowanie / Resultado zawsze na końcu.</t>
-  </si>
-  <si>
-    <t>ten Excel (opcjonalnie)</t>
-  </si>
-  <si>
     <t>comingSoon</t>
   </si>
   <si>
-    <t>Żebym mógł wciągnąć teksty z folderu</t>
-  </si>
-  <si>
     <t>true = Coming soon (wyszarzone), false = aktywny. Tylko EN.</t>
   </si>
   <si>
-    <t>CAPS (etykiety, tytuły, info) robi CSS na stronie — w Excelu pisz normalnie. Nawiasów [ ] przy labelach nie dopisuj.</t>
-  </si>
-  <si>
     <t>categories</t>
   </si>
   <si>
@@ -149,9 +155,6 @@
     <t>Filtry strony: ux-ui, motion, ai-engineering, development, branding (po przecinku). Tylko EN.</t>
   </si>
   <si>
-    <t>Pola tylko EN (żółte i tak wypełnij w kolumnie EN)</t>
-  </si>
-  <si>
     <t>Karta</t>
   </si>
   <si>
@@ -162,9 +165,6 @@
   </si>
   <si>
     <t>Now identyfikacja dla Epic Realty</t>
-  </si>
-  <si>
-    <t>slug, folderName, order, comingSoon, categories, year, liveUrl.</t>
   </si>
   <si>
     <t>Nuevo imagen de Epic Realty</t>
@@ -414,22 +414,19 @@
     <t>sections.1.text</t>
   </si>
   <si>
-    <t>We kicked off with a collaborative Brand Sprint to define core brand pillars and map out the target buyer persona. Based on those strategic insights, I crafted a visual framework built on three key pillars:
-- Custom Typography &amp; Multi-Layered Symbolism: I designed a custom sans-serif logotype featuring precise, bespoke letterform cuts for the Epic Realty wordmark. Complementing it is a geometric mark enclosed in a cylindrical circle, weaving together four distinct meanings: sun rays (Panama’s tropical luxury), a human silhouette (the founders' hands-on client service), a vertical pillar (financial stability), and a subtle roofline (the core real estate focus). The mark was engineered for total versatility—functioning seamlessly as a full logo, a standalone emblem, or in high-contrast monochrome.
-- Evolving the Color Palette: I modernized the traditional, heavy dark green palette. By combining a refined forest green with a softer, pastel-green accent, we retained a high-end feel while infusing much-needed freshness and agility into the brand.
-- Brutalist Supporting Typography: To set Epic Realty apart from local competitors, I introduced Barlow Condensed as the primary secondary typeface for marketing collateral and social media. Its architectural, semi-brutalist structure breaks away from traditional real estate tropes, giving the brand a bold, contemporary edge.</t>
-  </si>
-  <si>
-    <t>Współpracę rozpoczęliśmy od wspólnych warsztatów strategicznych (Brand Sprint), podczas których zdefiniowaliśmy filary marki i przeanalizowaliśmy profil zamożnego klienta końcowego. Na tej podstawie opracowałem kompleksową strategię wizualną opartą na trzech głównych filarach:
-- Autorska Typografia i Multi-Symbolika: Zaprojektowałem skustomizowany, bezszeryfowy logotyp z unikalnymi, precyzyjnymi cięciami w literach napisu Epic Realty. Dopełnieniem stał się geometryczny sygnet wpisany w kształt cylindrycznego koła, który łączy w sobie cztery symboliczne znaczenia: promienie słoneczne (luksusowy klimat Panamy), sylwetkę człowieka (personalne podejście founderów), pionowy filar (stabilność inwestycji) oraz zarys dachu (sektor nieruchomości). Znak przygotowałem tak, by działał bezprzegrodowo jako monolit, niezależny sygnet czy w wersji monochromatycznej.
-- Ewolucja Palety Barw: Przełamałem ciężki, archaiczny charakter tradycyjnej zieleni. Główną, szlachetną zieleń zestawioną z kontrastowym, jaśniejszym pastelowo-zielonym akcentem poddałem stonowaniu. Utrzymanie pastelowego wykończenia pozwoliło zachować luksusowy ton, dodając jej jednocześnie pożądanej świeżości i nowoczesności.
-- Brutalistyczna Typografia Komplementarna: Aby całkowicie odróżnić markę od konkurencji, do komunikacji w mediach społecznościowych wprowadziłem krój Barlow Condensed. Jego architektoniczny, lekko brutalistyczny wydźwięk nadał komunikacji nowoczesnej dynamiki i przełamał utarte schematy rynkowe.</t>
-  </si>
-  <si>
-    <t>Iniciamos el proceso con un Brand Sprint estratégico para definir los pilares de la marca y analizar a detalle al cliente ideal. A partir de esos hallazgos, desarrollé un sistema visual fundamentado en tres ejes:
-- Tipografía Personalizada y Simbolismo Multinivel: Diseñé un logotipo sans-serif a medida con cortes geométricos precisos en cada letra. Como complemento, creé un isotipo inscrito en una forma circular cilíndrica que integra cuatro significados clave: destellos solares (el lujo tropical de Panamá), una silueta humana (la atención personal de los fundadores), una columna vertical (la solidez de las inversiones) y la línea sutil de un techo (el sector inmobiliario). El símbolo fue estructurado para funcionar con total versatilidad: como logotipo completo, como isotipo independiente o en versiones monocromáticas.
-- Evolución de la Paleta de Color: Modernizamos el verde oscuro tradicional mediante tonos más suaves y matices pastel. Al combinar un verde bosque profundo con un acento verde pastel más luminoso, conservamos la elegancia propia del sector de lujo pero aportando mayor ligereza y dinamismo visual.
-- Tipografía Secundaria de Impacto: Para desmarcar a la firma de la competencia, introduje la tipografía Barlow Condensed para piezas editoriales y redes sociales. Su estructura arquitectónica y ligeramente brutalista rompe con los clichés inmobiliarios habituales, dándole a la comunicación de la marca un carácter firme y contemporáneo.</t>
+    <t>We kicked off with a collaborative Brand Sprint to define core brand pillars and map out the target buyer persona. Based on those strategic insights, I crafted a cohesive visual direction centered on custom typography, purposeful iconography, and a refined color balance.
+For the primary identity, I designed a custom sans-serif logotype featuring precise, bespoke letterform cuts for the Epic Realty wordmark. Complementing it is a geometric mark enclosed in a cylindrical circle, weaving together four distinct meanings: sun rays reflecting Panama’s tropical luxury, a human silhouette representing the founders' hands-on advisory approach, a vertical pillar symbolizing financial stability, and a subtle roofline defining the real estate focus. The mark was engineered for total versatility, functioning seamlessly as a full logo, a standalone emblem, or in high-contrast monochrome.
+To modernize the visual tone, I evolved the traditional dark green palette by introducing a softer, pastel-green accent alongside the refined forest green, retaining a high-end feel while infusing fresh energy into the brand. Additionally, to set Epic Realty apart from local competitors, I selected Barlow Condensed as the primary supporting typeface for marketing collateral and social channels. Its architectural, semi-brutalist structure breaks away from traditional real estate tropes, giving the brand a bold, contemporary edge.</t>
+  </si>
+  <si>
+    <t>Współpracę rozpoczęliśmy od wspólnych warsztatów strategicznych (Brand Sprint), podczas których zdefiniowaliśmy filary marki i przeanalizowaliśmy profil zamożnego klienta końcowego. Na tej podstawie opracowałem kompleksową strategię wizualną opartą na autorskich rozwiązaniach typograficznych, przemyślanej symbolice oraz nowoczesnym operowaniu kolorem.
+W ramach prac nad nowym znakiem zaprojektowałem skustomizowany, bezszeryfowy logotyp z unikalnymi, precyzyjnymi cięciami w literach napisu Epic Realty. Dopełnieniem stał się geometryczny sygnet wpisany w kształt cylindrycznego koła, który łączy w sobie cztery symboliczne znaczenia: promienie słoneczne nawiązujące do luksusowego klimatu Panamy, sylwetkę człowieka akcentującą personalne podejście founderów, pionowy filar reprezentujący stabilność inwestycji oraz zarys dachu jednoznacznie definiujący sektor nieruchomości. Znak został przygotowany tak, by działał bezprzegrodowo jako monolit, niezależny sygnet czy w wariancie monochromatycznym.
+Równolegle przełamałem ciężki, archaiczny charakter tradycyjnej zieleni. Główną, szlachetną zieleń poddałem stonowaniu i zestawiłem z kontrastowym, jaśniejszym pastelowo-zielonym akcentem, co pozwoliło zachować luksusowy ton, dodając marce pożądanej świeżości. Aby całkowicie odróżnić firmę od konkurencji, do komunikacji w mediach społecznościowych wprowadziłem krój Barlow Condensed. Jego architektoniczny, lekko brutalistyczny wydźwięk nadał komunikacji nowoczesnej dynamiki i skutecznie przełamał utarte schematy rynkowe.</t>
+  </si>
+  <si>
+    <t>Iniciamos el proceso con un Brand Sprint estratégico para definir los pilares de la marca y analizar a detalle al cliente ideal. A partir de esos hallazgos, desarrollé un sistema visual unificado fundamentado en soluciones tipográficas personalizadas, un simbolismo consciente y una equilibrada evolución del color.
+Para el identificador principal, diseñé un logotipo sans-serif a medida con cortes geométricos precisos en cada letra. Como complemento, creé un isotipo inscrito en una forma circular cilíndrica que integra cuatro significados clave: destellos solares reflejando el lujo tropical de Panamá, una silueta humana representando el trato personal de los fundadores, una columna vertical expresando la solidez de las inversiones y la línea sutil de un techo definiendo el sector inmobiliario. El símbolo fue estructurado para funcionar con total versatilidad, ya sea como logotipo completo, como isotipo independiente o en versiones monocromáticas.
+A nivel cromático, modernizamos el verde oscuro tradicional mediante tonos más suaves y matices pastel, logrando un contraste entre un verde bosque profundo y un acento verde pastel que conserva la elegancia propia del segmento de lujo pero aporta mayor ligereza. Finalmente, para desmarcar a la firma de la competencia, introduje la tipografía Barlow Condensed para piezas editoriales y redes sociales, cuya estructura arquitectónica y ligeramente brutalista rompe con los clichés habituales y le da un carácter firme y contemporáneo a la marca.</t>
   </si>
   <si>
     <t>Sekcja 03</t>
@@ -986,7 +983,7 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -1016,7 +1013,7 @@
     </row>
     <row r="4" ht="39.75" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -1046,7 +1043,7 @@
     </row>
     <row r="5" ht="39.75" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -1076,7 +1073,7 @@
     </row>
     <row r="6" ht="39.75" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -1106,7 +1103,7 @@
     </row>
     <row r="7" ht="39.75" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -1136,7 +1133,7 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1166,7 +1163,7 @@
     </row>
     <row r="10" ht="39.75" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1196,7 +1193,7 @@
     </row>
     <row r="11" ht="39.75" customHeight="1">
       <c r="A11" s="5" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1226,7 +1223,7 @@
     </row>
     <row r="12" ht="39.75" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1256,7 +1253,7 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1286,7 +1283,7 @@
     </row>
     <row r="15" ht="39.75" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -2318,22 +2315,22 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
@@ -2361,15 +2358,15 @@
         <v>13</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D2" s="8"/>
       <c r="E2" s="9"/>
       <c r="F2" s="6" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
@@ -2397,19 +2394,19 @@
         <v>13</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
@@ -2437,19 +2434,19 @@
         <v>13</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
@@ -2477,19 +2474,19 @@
         <v>13</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C5" s="16" t="b">
         <v>0</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
@@ -2517,19 +2514,19 @@
         <v>13</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
@@ -2554,16 +2551,16 @@
     </row>
     <row r="7" ht="24.0" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E7" s="18" t="s">
         <v>50</v>
@@ -2594,7 +2591,7 @@
     </row>
     <row r="8" ht="31.5" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>52</v>
@@ -2960,13 +2957,13 @@
         <v>86</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>87</v>
@@ -3000,13 +2997,13 @@
         <v>88</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E18" s="24" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>89</v>
@@ -3400,13 +3397,13 @@
         <v>135</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>110</v>
@@ -3440,13 +3437,13 @@
         <v>136</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F29" s="6" t="s">
         <v>115</v>
@@ -3480,13 +3477,13 @@
         <v>137</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>120</v>
@@ -3520,13 +3517,13 @@
         <v>139</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F31" s="6" t="s">
         <v>110</v>
@@ -3560,13 +3557,13 @@
         <v>140</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>115</v>
@@ -3600,13 +3597,13 @@
         <v>141</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F33" s="6" t="s">
         <v>120</v>
@@ -3640,13 +3637,13 @@
         <v>143</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>110</v>
@@ -3680,13 +3677,13 @@
         <v>144</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D35" s="21" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F35" s="6" t="s">
         <v>115</v>
@@ -3720,13 +3717,13 @@
         <v>145</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>120</v>
@@ -3760,13 +3757,13 @@
         <v>147</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D37" s="21" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F37" s="6" t="s">
         <v>110</v>
@@ -3800,13 +3797,13 @@
         <v>148</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>115</v>
@@ -3840,13 +3837,13 @@
         <v>149</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D39" s="21" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F39" s="6" t="s">
         <v>120</v>
@@ -3880,13 +3877,13 @@
         <v>151</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>110</v>
@@ -3920,13 +3917,13 @@
         <v>152</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D41" s="21" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F41" s="6" t="s">
         <v>115</v>
@@ -3960,13 +3957,13 @@
         <v>153</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>120</v>
@@ -5090,10 +5087,10 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -5122,7 +5119,7 @@
     </row>
     <row r="2" ht="27.75" customHeight="1">
       <c r="A2" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>12</v>
@@ -5218,10 +5215,10 @@
     </row>
     <row r="5" ht="27.75" customHeight="1">
       <c r="A5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>27</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -5282,7 +5279,7 @@
     </row>
     <row r="7" ht="27.75" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
Unify Epic Realty into single project, update category boxes to white badges, set permanent light mode on project sections, and add testimonial section
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/portfolio/epic-realty/Epic Realty.xlsx
+++ b/public/portfolio/epic-realty/Epic Realty.xlsx
@@ -4,170 +4,155 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Instrukcja" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Projekt" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Grafiki" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Tłumaczenia (PL - EN - ES)" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="Grafiki i media" sheetId="3" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">Projekt!$A$1:$F$45</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Tłumaczenia (PL - EN - ES)'!$A$1:$F$55</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="218">
+  <si>
+    <t>Chris Bartosik — Szablon projektu (Wersja: 2026-08-29)</t>
+  </si>
+  <si>
+    <t>Plik w folderze public/portfolio/{folderName}/</t>
+  </si>
+  <si>
+    <t>Sekcja</t>
+  </si>
+  <si>
+    <t>Rola pliku na stronie</t>
+  </si>
+  <si>
+    <t>Klucz pola</t>
+  </si>
+  <si>
+    <t>Polski (PL)</t>
+  </si>
+  <si>
+    <t>Angielski (EN)</t>
+  </si>
+  <si>
+    <t>Hiszpański (ES)</t>
+  </si>
+  <si>
+    <t>Instrukcja / Uwagi</t>
+  </si>
+  <si>
+    <t>Data wygenerowania szablonu: 29.08.2026</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>Jak używać:</t>
+  </si>
+  <si>
+    <t>cover.webp / cover.webm / cover.mp4</t>
+  </si>
+  <si>
+    <t>slug</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Okładka / wideo na liście projektów</t>
+  </si>
+  <si>
+    <t>Nazwa pliku projektu, np. epic-realty (→ epic-realty.md). Tylko EN.</t>
+  </si>
+  <si>
+    <t>bg.webp</t>
+  </si>
+  <si>
+    <t>Tło w sekcji Hero na stronie projektu</t>
+  </si>
+  <si>
+    <t>1. Skopiuj plik i nazwij np. [NazwaProjektu].xlsx (jeden Excel = jeden projekt).</t>
+  </si>
+  <si>
+    <t>folderName</t>
+  </si>
+  <si>
+    <t>Folder grafik: public/portfolio/{folderName}/. Zdjęcia bierze strona sama. Tylko EN.</t>
+  </si>
+  <si>
+    <t>1.webp</t>
+  </si>
+  <si>
+    <t>Grafika / media w sekcji Intro (opcjonalnie)</t>
+  </si>
+  <si>
+    <t>2. W karcie „Tłumaczenia (PL - EN - ES)” uzupełnij teksty dla 3 języków.</t>
+  </si>
+  <si>
+    <t>order</t>
+  </si>
+  <si>
+    <t>Kolejność na liście (1, 2, 3…). Mniejsza = wyżej. Tylko EN.</t>
+  </si>
+  <si>
+    <t>X.1.webp / X.1.mp4</t>
+  </si>
+  <si>
+    <t>Sekcja X: 1 duże zdjęcie / wideo na pełną szerokość</t>
+  </si>
+  <si>
+    <t>3. Sekcja 1 (Intro) oraz ostatnia sekcja (Summary) mają już wstępnie wpisane etykiety.</t>
+  </si>
+  <si>
+    <t>comingSoon</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>true = Coming soon (wyszarzone), false = aktywny. Tylko EN.</t>
+  </si>
+  <si>
+    <t>4. Na samym dole znajduje się opcjonalna sekcja „Opinia klienta” (cytat, autor, stanowisko).</t>
+  </si>
+  <si>
+    <t>X.2.webp + X.3.webp</t>
+  </si>
+  <si>
+    <t>Sekcja X: 2 mniejsze zdjęcia (w parze obok siebie 50%/50%)</t>
+  </si>
+  <si>
+    <t>categories</t>
+  </si>
+  <si>
+    <t>branding, ux-ui, webflow</t>
+  </si>
+  <si>
+    <t>5. Wrzuć grafiki do folderu public/portfolio/{folderName}/ (cover, bg, X.1, X.2, X.3, X.4).</t>
+  </si>
+  <si>
+    <t>Filtry strony: ux-ui, motion, ai-engineering, development, branding (po przecinku). Tylko EN.</t>
+  </si>
+  <si>
+    <t>X.4.webp / X.4.mp4</t>
+  </si>
+  <si>
+    <t>Karta</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>Zasady automatyczne (nie wpisujesz w Excelu):</t>
+  </si>
   <si>
     <t>Epic Realty</t>
   </si>
   <si>
-    <t>Wrzucasz do folderu projektu</t>
-  </si>
-  <si>
-    <t>Sekcja</t>
-  </si>
-  <si>
-    <t>Co robi</t>
-  </si>
-  <si>
-    <t>Pole</t>
-  </si>
-  <si>
-    <t>EN</t>
-  </si>
-  <si>
-    <t>PL</t>
-  </si>
-  <si>
-    <t>Jak używać</t>
-  </si>
-  <si>
-    <t>ES</t>
-  </si>
-  <si>
-    <t>Uwagi</t>
-  </si>
-  <si>
-    <t>1. Skopiuj plik i nazwij np. Epic Realty.xlsx (jeden Excel = jeden projekt).</t>
-  </si>
-  <si>
-    <t>cover.webp / cover.webm / cover.mp4</t>
-  </si>
-  <si>
-    <t>Okładka na liście projektów</t>
-  </si>
-  <si>
-    <t>Start</t>
-  </si>
-  <si>
-    <t>2. W karcie „Projekt” uzupełnij EN, PL i ES — tylko teksty.</t>
-  </si>
-  <si>
-    <t>slug</t>
-  </si>
-  <si>
-    <t>epic-realty</t>
-  </si>
-  <si>
-    <t>bg.webp</t>
-  </si>
-  <si>
-    <t>Tło hero na stronie projektu</t>
-  </si>
-  <si>
-    <t>3. Wrzuć grafiki do public/portfolio/{folderName}/ (cover, bg, 1.webp, 2.webp…).</t>
-  </si>
-  <si>
-    <t>4. Wyślij mi Excel albo wrzuć go do tego folderu — ja wciągam treści.</t>
-  </si>
-  <si>
-    <t>1.webp</t>
-  </si>
-  <si>
-    <t>Grafika przy Overview (opcjonalnie)</t>
-  </si>
-  <si>
-    <t>Nazwa pliku projektu, np. epic-realty (→ epic-realty.md). Tylko EN.</t>
-  </si>
-  <si>
-    <t>Co jest automatyczne (nie wpisujesz w Excelu)</t>
-  </si>
-  <si>
-    <t>2.webp, 3.webp, 4.webp…</t>
-  </si>
-  <si>
-    <t>Pełne kadry w galerii (kolejność = numer)</t>
-  </si>
-  <si>
-    <t>Zdjęcia i wideo: cover.webp/mp4, bg.webp, 1.webp (overview), 2.webp / 2.1+2.2… — strona czyta je z folderu. Nie ma pól afterGroup / ścieżek grafik.</t>
-  </si>
-  <si>
-    <t>folderName</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Układ i kolory sekcji: theme idzie automatycznie (dark → light → muted). Overview zawsze jasny. Sekcja Summary / Podsumowanie / Resultado zawsze na końcu.</t>
-  </si>
-  <si>
-    <t>2.1.webp + 2.2.webp…</t>
-  </si>
-  <si>
-    <t>Pary pod pełnym kadrem o tym samym numerze</t>
-  </si>
-  <si>
-    <t>CAPS (etykiety, tytuły, info) robi CSS na stronie — w Excelu pisz normalnie. Nawiasów [ ] przy labelach nie dopisuj.</t>
-  </si>
-  <si>
-    <t>Folder grafik: public/portfolio/{folderName}/. Zdjęcia bierze strona sama. Tylko EN.</t>
-  </si>
-  <si>
-    <t>Pola tylko EN (żółte i tak wypełnij w kolumnie EN)</t>
-  </si>
-  <si>
-    <t>order</t>
-  </si>
-  <si>
-    <t>ten Excel (opcjonalnie)</t>
-  </si>
-  <si>
-    <t>Żebym mógł wciągnąć teksty z folderu</t>
-  </si>
-  <si>
-    <t>slug, folderName, order, comingSoon, categories, year, liveUrl.</t>
-  </si>
-  <si>
-    <t>Kolejność na liście (1, 2, 3…). Mniejsza = wyżej. Tylko EN.</t>
-  </si>
-  <si>
-    <t>comingSoon</t>
-  </si>
-  <si>
-    <t>true = Coming soon (wyszarzone), false = aktywny. Tylko EN.</t>
-  </si>
-  <si>
-    <t>categories</t>
-  </si>
-  <si>
-    <t>Branding</t>
-  </si>
-  <si>
-    <t>Filtry strony: ux-ui, motion, ai-engineering, development, branding (po przecinku). Tylko EN.</t>
-  </si>
-  <si>
-    <t>Karta</t>
-  </si>
-  <si>
-    <t>title</t>
-  </si>
-  <si>
-    <t>New identity for Epic Realty</t>
-  </si>
-  <si>
-    <t>Now identyfikacja dla Epic Realty</t>
-  </si>
-  <si>
-    <t>Nuevo imagen de Epic Realty</t>
+    <t>Grafiki i wideo: strona pobiera je automatycznie z folderu projektu według schematu X.1, X.2, X.3, X.4.</t>
   </si>
   <si>
     <t>Tytuł na liście projektów i w przeglądarce.</t>
@@ -176,12 +161,15 @@
     <t>category</t>
   </si>
   <si>
-    <t>Rebranding</t>
+    <t>Kolorystyka sekcji: sekcje 2, 4, 6, 8 automatycznie mają ciemne tło (dark mode), a Intro i Summary zawsze białe.</t>
   </si>
   <si>
     <t>Krótka kategoria pod tytułem (np. Rebranding). Tłumacz w PL/ES jeśli trzeba.</t>
   </si>
   <si>
+    <t>Wielkie litery (CAPS): formatowane są automatycznie przez styl strony — w Excelu pisz naturalnie.</t>
+  </si>
+  <si>
     <t>Hero</t>
   </si>
   <si>
@@ -194,12 +182,12 @@
     <t>clientLabel</t>
   </si>
   <si>
+    <t>Klient</t>
+  </si>
+  <si>
     <t>Client</t>
   </si>
   <si>
-    <t>Klient</t>
-  </si>
-  <si>
     <t>Cliente</t>
   </si>
   <si>
@@ -209,13 +197,13 @@
     <t>heroSubtitle</t>
   </si>
   <si>
-    <t>Rebranding for a luxury real estate studio from Panama</t>
-  </si>
-  <si>
-    <t>Rebranding luksusowego studia nieruchomości w Panamie</t>
-  </si>
-  <si>
-    <t>Rebranding para Agencia Inmobiliaria de Lujo en Panamá</t>
+    <t>Cyfrowa i wizerunkowa transformacja luksusowej agencji nieruchomości w Panamie.</t>
+  </si>
+  <si>
+    <t>Elevating Panama's premier boutique real estate agency through brand identity and digital design.</t>
+  </si>
+  <si>
+    <t>Transformando la presencia de la agencia inmobiliaria boutique más exclusiva de Panamá.</t>
   </si>
   <si>
     <t>Podtytuł pod klientem. Enter = nowa linia na stronie.</t>
@@ -227,13 +215,13 @@
     <t>service</t>
   </si>
   <si>
-    <t>Logo design, Rebranding</t>
-  </si>
-  <si>
-    <t>Design loga, Rebranding</t>
-  </si>
-  <si>
-    <t>Diseño de Logo, Rebranding</t>
+    <t>identyfikacja wizualna, web design, wdrożenie webflow, cms</t>
+  </si>
+  <si>
+    <t>brand identity, web design, webflow development, cms</t>
+  </si>
+  <si>
+    <t>identidad de marca, diseño web, desarrollo webflow, cms</t>
   </si>
   <si>
     <t>Puste = ukryte na stronie.</t>
@@ -242,13 +230,13 @@
     <t>industry</t>
   </si>
   <si>
-    <t>Real estate, Luxury</t>
-  </si>
-  <si>
-    <t>Nieruchomości, Luksusowe</t>
-  </si>
-  <si>
-    <t>Bienes Raíces, Sector de Lujo</t>
+    <t>Nieruchomości Premium, Inwestycje</t>
+  </si>
+  <si>
+    <t>Luxury Real Estate, Investments</t>
+  </si>
+  <si>
+    <t>Bienes Raíces de Lujo, Inversiones</t>
   </si>
   <si>
     <t>market</t>
@@ -263,13 +251,16 @@
     <t>tools</t>
   </si>
   <si>
-    <t>Figma, Adobe</t>
+    <t>Figma, Webflow</t>
   </si>
   <si>
     <t>year</t>
   </si>
   <si>
-    <t>Rok, np. 2025. Tylko EN.</t>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>Rok, np. 2026. Tylko EN.</t>
   </si>
   <si>
     <t>Live</t>
@@ -287,7 +278,7 @@
     <t>Adres URL. Tylko EN. Puste = bez linku.</t>
   </si>
   <si>
-    <t>Overview</t>
+    <t>Overview / Sekcja 01</t>
   </si>
   <si>
     <t>overviewLabel</t>
@@ -296,41 +287,37 @@
     <t>Intro</t>
   </si>
   <si>
-    <t>Introducción</t>
-  </si>
-  <si>
-    <t>Etykieta bez [ ]. Puste = Overview / Kontekst / Descripción.</t>
+    <t>Etykieta 1. sekcji (Intro/Overview). Puste = domyślne [Intro] / [Kontekst] / [Descripción].</t>
   </si>
   <si>
     <t>overviewTitle</t>
   </si>
   <si>
-    <t>A fresh, high-end visual identity for a Panamanian boutique real estate agency.</t>
-  </si>
-  <si>
-    <t>Nowy, profesjonalny wizerunek dla panamskiej agencji nieruchomości z sektora premium.</t>
-  </si>
-  <si>
-    <t>Una nueva imagen de alto nivel para una firma boutique en el mercado inmobiliario panameño.</t>
-  </si>
-  <si>
-    <t>Nagłówek bloku overview.</t>
+    <t>Butikowy lider w segmencie nieruchomości premium w Panamie</t>
+  </si>
+  <si>
+    <t>Setting a New Benchmark in Panama's High-End Real Estate Market</t>
+  </si>
+  <si>
+    <t>Redefiniendo el concepto de bienes raíces de lujo en Panamá</t>
+  </si>
+  <si>
+    <t>Nagłówek bloku overview / intro.</t>
   </si>
   <si>
     <t>overviewText</t>
   </si>
   <si>
-    <t>Epic Realty is a boutique real estate agency based in Panama, specializing in multi-million dollar luxury investments. The founders approached me to execute a complete rebranding. Their legacy logo—created during the company’s early bootstrapped phase—lacked typographic precision and technical polish. It failed to convey the exclusivity of their property portfolio and couldn't build the necessary authority with high-net-worth investors.</t>
-  </si>
-  <si>
-    <t>Epic Realty to luksusowe studio nieruchomości z Panamy, specjalizujące się w obsłudze inwestycji z najwyższej półki cenowej — transakcji sięgających portfeli wielomilionowych. Założyciele marki zgłosili się do mnie z potrzebą przeprowadzenia kompletnego rebrandingu. Ich dotychczasowa identyfikacja, stworzona na wczesnym, budżetowym etapie rozwoju firmy, była niepoprawna pod kątem sztuki typograficznej i technicznej. Znak nie oddawał ekskluzywnego charakteru oferowanych nieruchomości ani nie budował odpowiedniego prestiżu w oczach zamożnych inwestorów z sektora High-Net-Worth.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Epic Realty es una agencia boutique de bienes raíces en Panamá especializada en propiedades exclusivas e inversiones multimillonarias. Sus fundadores me contactaron con la necesidad de ejecutar un rebranding integral. Su identidad anterior, desarrollada en la etapa inicial de la empresa, carecía de precisión tipográfica y refinamiento técnico, por lo que no proyectaba el nivel de exclusividad de su portafolio ni generaba la confianza necesaria ante inversionistas de alto patrimonio.
-</t>
-  </si>
-  <si>
-    <t>Treść. Pusta linia = nowy akapit.</t>
+    <t>Epic Realty to butikowa agencja nieruchomości premium, która operuje w najbardziej prestiżowych lokalizacjach Panamy. Marka zbudowała swoją pozycję na bezkompromisowej zasadzie „jakość, a nie ilość” — zamiast masowego katalogu ofert, selekcjonuje wyłącznie unikalne rezydencje, penthouse'y i luksusowe apartamenty. Jej fundamentem jest indywidualne podejście do klienta, wysoka kultura relacji oraz głębokie zrozumienie architektury najwyższej próby. Moim zadaniem przy tej współpracy było pełne zdefiniowanie tożsamości Epic Realty na nowo, odświeżenie jej wizualnego, profesjonalnego sznytu oraz stworzenie cyfrowego doświadczenia i platformy internetowej, które pozwalają marce wybić się na tle konkurencji i dominować na panamskim rynku nieruchomości luksusowych.</t>
+  </si>
+  <si>
+    <t>Epic Realty is an exclusive boutique real estate firm operating across Panama’s most sought-after addresses. Rejecting volume-driven market practices, the agency adheres strictly to a 'quality over quantity' philosophy, curating a tight portfolio of high-end residences, penthouses, and architectural landmarks. Built on hyper-personalized client service and deep market discretion, Epic needed a brand experience to match its reputation. My objective in this collaboration was to rethink their entire visual identity, refresh their professional presence, and build a digital platform that positions them as the undisputed leader in local luxury real estate.</t>
+  </si>
+  <si>
+    <t>Epic Realty es una firma inmobiliaria boutique especializada en las propiedades más exclusivas de Panamá. Guiada por la premisa de 'calidad sobre cantidad', la agencia evita los catálogos masivos para enfocarse en una selección impecable de residencias de autor, penthouses y apartamentos de lujo. Con un enfoque basado en el trato personalizado y el conocimiento profundo de la arquitectura de alta gama, mi objetivo en esta colaboración fue redefinir por completo su identidad de marca, renovar su carácter profesional y construir una plataforma web a la altura de su portafolio.</t>
+  </si>
+  <si>
+    <t>Treść intro. Pusta linia = nowy akapit.</t>
   </si>
   <si>
     <t>Sekcja 01</t>
@@ -339,28 +326,25 @@
     <t>sections.0.label</t>
   </si>
   <si>
-    <t>CHALLENGE</t>
-  </si>
-  <si>
-    <t>WYZWANIE</t>
-  </si>
-  <si>
-    <t>Desafío</t>
-  </si>
-  <si>
-    <t>Etykieta bez [ ], np. Challenge / Wyzwanie. Puste = sekcja nieużywana.</t>
+    <t>Research &amp; Brand Sprint</t>
+  </si>
+  <si>
+    <t>Investigación y Brand Sprint</t>
+  </si>
+  <si>
+    <t>Etykieta bez [ ], np. Challenge / Strategy / Design. Puste = sekcja nieużywana.</t>
   </si>
   <si>
     <t>sections.0.title</t>
   </si>
   <si>
-    <t>Blending classic prestige with modern digital flair to stand out in a crowded market.</t>
-  </si>
-  <si>
-    <t>Połączenie tradycyjnej elegancji z nowoczesnym stylem i wyróżnienie się na przebodźcowanym rynku.</t>
-  </si>
-  <si>
-    <t>Fusionar la elegancia tradicional con un estilo contemporáneo y destacar en un mercado saturado.</t>
+    <t>Luki wizerunkowe i generyczne szablony konkurencji</t>
+  </si>
+  <si>
+    <t>Uncovering Visual Clichés in a Template-Driven Market</t>
+  </si>
+  <si>
+    <t>Superando la monotonía visual del sector inmobiliario local</t>
   </si>
   <si>
     <t>Nagłówek sekcji.</t>
@@ -369,19 +353,16 @@
     <t>sections.0.text</t>
   </si>
   <si>
-    <t>The core challenge was balancing two contrasting founder visions: capturing the heritage and weight of classic luxury brands (drawing inspiration from Rolex’s aesthetic and signature green) while delivering a clean, contemporary presence tailored for digital touchpoints.
-Furthermore, Panama's real estate market was saturated with generic serif fonts and dated italics. We needed to cut through the industry noise with a visual identity that radiates trust, highlights the founders' personal advisory approach, and captures attention across social channels.</t>
-  </si>
-  <si>
-    <t>Głównym wyzwaniem projektowym było umiejętne pogodzenie dwóch z pozoru odmiennych wizji założycieli: chęci nawiązania do tradycyjnych, konserwatywnych marek luksusowych (punktem odniesienia była dla nich m.in. estetyka marki Rolex i ich szlachetna zieleń) z potrzebą wyrazistej, współczesnej i unikalnej prezentacji w przestrzeni cyfrowej.
-Dodatkowo rynek nieruchomości w Panamie okazał się niezwykle przeładowany powtarzalnymi schematami – większość konkurencyjnych agencji korzystała z generycznych krojów szeryfowych lub klasycznych kursyw. Musieliśmy przełamać ten rynkowy szum i stworzyć język wizualny, który zbuduje natychmiastowe zaufanie inwestorów, odda personalne podejście founderów, a jednocześnie wyróżni markę w kanałach social media.</t>
-  </si>
-  <si>
-    <t>El reto central consistió en equilibrar dos visiones aparentemente opuestas de los fundadores: evocar el prestigio de las marcas de lujo tradicionales (tomando como referencia la estética de Rolex y su característico tono verde) sin perder la frescura y relevancia visual en entornos digitales.
-Además, el sector inmobiliario en Panamá suele caer en patrones muy repetitivos, abusando de tipografías serif genéricas e itálicas convencionales. El desafío fue romper con esa inercia y crear un lenguaje gráfico que transmitiera confianza inmediata, reflejara el trato personalizado de los socios y marcara la diferencia en canales digitales.</t>
-  </si>
-  <si>
-    <t>Treść. Listy: - **Tytuł**: opis. Puste = sekcja nieużywana.</t>
+    <t>Prace rozpoczęliśmy od warsztatu Brand Sprint przeprowadzonego bezpośrednio z założycielami Epic Realty. Wykorzystując metodologię Golden Circle, precyzyjnie sformułowaliśmy misję marki opartą na podnoszeniu standardów doradztwa na panamskim rynku nieruchomości luksusowych poprzez autentyczność, bezwzględną dyskrecję i wiedzę architektoniczną. Ten etap pozwolił nam zdefiniować osobowość Epic jako przemyślane zestawienie dojrzałości, elegancji, strategicznego myślenia i nuty śmiałości, co stało się fundamentem do odrzucenia bezosobowych praktyk sprzedażowych. Aby upewnić się, jak ten archetyp wypada na tle otoczenia, przeprowadziłem dokładny audyt konkurencji, który ujawnił dominację generycznych, pozbawionych wyrazu szablonów. Co więcej, dotychczasowa strona klienta na WordPressie cierpiała na chaos strukturalny, co utrudniało zarządzanie ofertami i znacząco osłabiało odbiór marki premium.</t>
+  </si>
+  <si>
+    <t>We kicked off the project with an intensive Brand Sprint workshop alongside Epic Realty’s founders. Using Simon Sinek’s Golden Circle framework, we defined the company’s core mission around elevating luxury real estate standards in Panama through genuine relationships, absolute discretion, and architectural expertise. This process allowed us to shape the brand personality as a thoughtful blend of maturity, elegance, strategic insight, and a touch of boldness, laying a strong foundation to reject impersonal sales tactics. To validate this direction, I conducted a thorough competitive audit that revealed a local market dominated by generic templates. On top of that, Epic’s legacy WordPress site suffered from structural chaos, making listing management frustrating and significantly weakening their high-end market positioning.</t>
+  </si>
+  <si>
+    <t>Iniciamos el proyecto liderando un taller de Brand Sprint junto a los fundadores de Epic Realty. Basándonos en la metodología del Círculo Dorado, definimos la misión central de la empresa enfocada en elevar los estándares del mercado inmobiliario de lujo en Panamá mediante relaciones auténticas, discreción absoluta y criterio arquitectónico. Este proceso nos permitió estructurar la personalidad de Epic como una combinación madura de elegancia, visión estratégica y un toque de audacia, sentando las bases para alejarnos de los enfoques comerciales impersonales. Para validar esta dirección, llevé a cabo un análisis competitivo que reveló un mercado dominado por plantillas genéricas. Además, el sitio anterior de Epic en WordPress presentaba un caos estructural que dificultaba la gestión de propiedades y debilitaba su posicionamiento premium.</t>
+  </si>
+  <si>
+    <t>Treść. Pusta linia = nowy akapit. Puste pole = sekcja nieużywana.</t>
   </si>
   <si>
     <t>Sekcja 02</t>
@@ -390,43 +371,37 @@
     <t>sections.1.label</t>
   </si>
   <si>
-    <t>STRATEGY</t>
-  </si>
-  <si>
-    <t>STRATEGIA</t>
-  </si>
-  <si>
-    <t>Estrategia</t>
+    <t>Wyzwanie Identyfikacyjne</t>
+  </si>
+  <si>
+    <t>Brand Identity Challenge</t>
+  </si>
+  <si>
+    <t>El desafío de la identidad</t>
   </si>
   <si>
     <t>sections.1.title</t>
   </si>
   <si>
-    <t>Bespoke typography, a multi-layered emblem, and bold visual choices.</t>
-  </si>
-  <si>
-    <t>Autorski logotyp, wielowarstwowy sygnet i odważny wybór typografii do komunikacji.</t>
-  </si>
-  <si>
-    <t>Tipografía a medida, un isotipo con narrativa propia y una dirección gráfica brutal.</t>
+    <t>Ewolucja od nieczytelnej formy do pełnego ekosystemu</t>
+  </si>
+  <si>
+    <t>From Legibility Issues to an Adaptive Ecosystem</t>
+  </si>
+  <si>
+    <t>Evolución de un formato ilegible a un sistema adaptable</t>
   </si>
   <si>
     <t>sections.1.text</t>
   </si>
   <si>
-    <t>We kicked off with a collaborative Brand Sprint to define core brand pillars and map out the target buyer persona. Based on those strategic insights, I crafted a cohesive visual direction centered on custom typography, purposeful iconography, and a refined color balance.
-For the primary identity, I designed a custom sans-serif logotype featuring precise, bespoke letterform cuts for the Epic Realty wordmark. Complementing it is a geometric mark enclosed in a cylindrical circle, weaving together four distinct meanings: sun rays reflecting Panama’s tropical luxury, a human silhouette representing the founders' hands-on advisory approach, a vertical pillar symbolizing financial stability, and a subtle roofline defining the real estate focus. The mark was engineered for total versatility, functioning seamlessly as a full logo, a standalone emblem, or in high-contrast monochrome.
-To modernize the visual tone, I evolved the traditional dark green palette by introducing a softer, pastel-green accent alongside the refined forest green, retaining a high-end feel while infusing fresh energy into the brand. Additionally, to set Epic Realty apart from local competitors, I selected Barlow Condensed as the primary supporting typeface for marketing collateral and social channels. Its architectural, semi-brutalist structure breaks away from traditional real estate tropes, giving the brand a bold, contemporary edge.</t>
-  </si>
-  <si>
-    <t>Współpracę rozpoczęliśmy od wspólnych warsztatów strategicznych (Brand Sprint), podczas których zdefiniowaliśmy filary marki i przeanalizowaliśmy profil zamożnego klienta końcowego. Na tej podstawie opracowałem kompleksową strategię wizualną opartą na autorskich rozwiązaniach typograficznych, przemyślanej symbolice oraz nowoczesnym operowaniu kolorem.
-W ramach prac nad nowym znakiem zaprojektowałem skustomizowany, bezszeryfowy logotyp z unikalnymi, precyzyjnymi cięciami w literach napisu Epic Realty. Dopełnieniem stał się geometryczny sygnet wpisany w kształt cylindrycznego koła, który łączy w sobie cztery symboliczne znaczenia: promienie słoneczne nawiązujące do luksusowego klimatu Panamy, sylwetkę człowieka akcentującą personalne podejście founderów, pionowy filar reprezentujący stabilność inwestycji oraz zarys dachu jednoznacznie definiujący sektor nieruchomości. Znak został przygotowany tak, by działał bezprzegrodowo jako monolit, niezależny sygnet czy w wariancie monochromatycznym.
-Równolegle przełamałem ciężki, archaiczny charakter tradycyjnej zieleni. Główną, szlachetną zieleń poddałem stonowaniu i zestawiłem z kontrastowym, jaśniejszym pastelowo-zielonym akcentem, co pozwoliło zachować luksusowy ton, dodając marce pożądanej świeżości. Aby całkowicie odróżnić firmę od konkurencji, do komunikacji w mediach społecznościowych wprowadziłem krój Barlow Condensed. Jego architektoniczny, lekko brutalistyczny wydźwięk nadał komunikacji nowoczesnej dynamiki i skutecznie przełamał utarte schematy rynkowe.</t>
-  </si>
-  <si>
-    <t>Iniciamos el proceso con un Brand Sprint estratégico para definir los pilares de la marca y analizar a detalle al cliente ideal. A partir de esos hallazgos, desarrollé un sistema visual unificado fundamentado en soluciones tipográficas personalizadas, un simbolismo consciente y una equilibrada evolución del color.
-Para el identificador principal, diseñé un logotipo sans-serif a medida con cortes geométricos precisos en cada letra. Como complemento, creé un isotipo inscrito en una forma circular cilíndrica que integra cuatro significados clave: destellos solares reflejando el lujo tropical de Panamá, una silueta humana representando el trato personal de los fundadores, una columna vertical expresando la solidez de las inversiones y la línea sutil de un techo definiendo el sector inmobiliario. El símbolo fue estructurado para funcionar con total versatilidad, ya sea como logotipo completo, como isotipo independiente o en versiones monocromáticas.
-A nivel cromático, modernizamos el verde oscuro tradicional mediante tonos más suaves y matices pastel, logrando un contraste entre un verde bosque profundo y un acento verde pastel que conserva la elegancia propia del segmento de lujo pero aporta mayor ligereza. Finalmente, para desmarcar a la firma de la competencia, introduje la tipografía Barlow Condensed para piezas editoriales y redes sociales, cuya estructura arquitectónica y ligeramente brutalista rompe con los clichés habituales y le da un carácter firme y contemporáneo a la marca.</t>
+    <t>Zidentyfikowane w trakcie audytu słabości dotyczyły również warstwy identyfikacji, gdzie dotychczasowe logo stwarzało poważne problemy w codziennej eksploatacji. Jego cienkie, znikające linie i zachwiane proporcje uniemożliwiały czytelną skalowalność, a zachowawcza paleta barw mijała się z aspiracjami do segmentu luxury. W odpowiedzi na te wyzwania zaprojektowałem elastyczny ekosystem wizualny, który buduje profesjonalny wizerunek i działa niezawodnie we wszystkich punktach styku z marką. Miało to kluczowe znaczenie zwłaszcza na rynku panamskim, gdzie profile społecznościowe oraz komunikatory stanowią główny kanał pierwszego kontaktu, przez co wyrazisty avatar i uniwersalny monogram stały się równie istotne jak eleganckie materiały drukowane czy katalogi rezydencji.</t>
+  </si>
+  <si>
+    <t>The weaknesses identified during the audit extended directly to the visual identity, where the legacy logo posed severe operational challenges. Its ultra-thin lines and awkward proportions made it fall apart at smaller scales, while the muted color scheme felt completely out of touch with a luxury positioning. In response to these challenges, I built a flexible visual ecosystem that establishes a commanding presence across all touchpoints. This proved especially crucial in the Panamanian market, where social profiles and messaging apps act as the primary point of contact, making a sharp social avatar and icon just as vital as high-end printed brochures or real estate catalogs.</t>
+  </si>
+  <si>
+    <t>Las deficiencias detectadas durante el diagnóstico afectaban también a la identidad gráfica, donde el logotipo anterior mostraba serios problemas de aplicación. Sus trazos excesivamente finos y proporciones desequilibradas impedían una correcta escalabilidad, mientras que su paleta de colores no lograba reflejar el estándar del sector inmobiliario de alto nivel. Para resolver estas limitaciones, diseñé un ecosistema visual flexible que proyecta un alto nivel de profesionalismo en cada punto de contacto. Esto resultó clave en el contexto panameño, donde las redes sociales y la mensajería instantánea son la vía principal de descubrimiento, haciendo que un avatar legible sea tan determinante como el material impreso y los catálogos de propiedades.</t>
   </si>
   <si>
     <t>Sekcja 03</t>
@@ -435,48 +410,156 @@
     <t>sections.2.label</t>
   </si>
   <si>
+    <t>Strategia Wizualna</t>
+  </si>
+  <si>
+    <t>Visual Direction</t>
+  </si>
+  <si>
+    <t>Estrategia de diseño</t>
+  </si>
+  <si>
     <t>sections.2.title</t>
   </si>
   <si>
+    <t>Typografia Barlow Condensed i paleta luksusu</t>
+  </si>
+  <si>
+    <t>Editorial Brutalism Meets Timeless Sophistication</t>
+  </si>
+  <si>
+    <t>Elegancia atemporal con un toque moderno y estructurado</t>
+  </si>
+  <si>
     <t>sections.2.text</t>
   </si>
   <si>
+    <t>Konsekwencją przyjęcia nowego systemu wizualnego był świadomy wybór typografii oraz palety barw, które jednoznacznie odróżniają Epic Realty od konkurencji. Zamiast sięgać po zachowawcze kroje szeryfowe, postawiłem na nowoczesny font Barlow Condensed o architektonicznym profilu, który nadaje marce wyrazistość, równoważąc go czytelnym i przejrzystym fontem Lato w warstwie tekstowej. Dopełnieniem tej koncepcji stała się paleta kolorystyczna inspirowana naturą Panamy oraz dyskretną elegancją. Głębokie odcienie Woodland Green i Panama Night stworzyły solidne tło dla stonowanego akcentu Boutique Green i czystej bieli, nadając całości szlachetny, uporządkowany charakter.</t>
+  </si>
+  <si>
+    <t>Building directly on this refined identity, we made intentional choices in typography and color to distinctly set Epic Realty apart from its peers. Instead of defaulting to traditional luxury serifs, I chose Barlow Condensed for its bold architectural character, balancing it with Lato for clean and effortless body copy. The color strategy draws inspiration from Panama’s lush landscape and understated elegance. Rich tones of Woodland Green and Panama Night provide a grounded foundation, complemented by subtle Boutique Green accents and generous white space to deliver a clean, elevated feel.</t>
+  </si>
+  <si>
+    <t>Como continuación natural de este nuevo sistema visual, seleccionamos una tipografía y una paleta cromática capaces de diferenciar a Epic Realty de la competencia. En lugar de recurrir a las clásicas fuentes con serifa, opté por Barlow Condensed debido a su perfil arquitectónico y contemporáneo, equilibrándolo con la claridad de Lato para los textos principales. La estrategia de color se inspiró en la naturaleza panameña y en el lujo sobrio. Los tonos profundos Woodland Green y Panama Night aportan una base firme, mientras que los acentos en Boutique Green y el espacio en blanco brindan una estética limpia y sofisticada.</t>
+  </si>
+  <si>
     <t>Sekcja 04</t>
   </si>
   <si>
     <t>sections.3.label</t>
   </si>
   <si>
+    <t>Pozycjonowanie UX &amp; UI</t>
+  </si>
+  <si>
+    <t>UX &amp; UI Strategy</t>
+  </si>
+  <si>
+    <t>Diseño de experiencia (UX/UI)</t>
+  </si>
+  <si>
     <t>sections.3.title</t>
   </si>
   <si>
+    <t>Czysty layout, akcent na media i metrykę rynkową</t>
+  </si>
+  <si>
+    <t>Immersive Imagery Grounded in Clear Technical Metrics</t>
+  </si>
+  <si>
+    <t>Experiencia visual inmersiva respaldada por datos clave</t>
+  </si>
+  <si>
     <t>sections.3.text</t>
   </si>
   <si>
+    <t>Ta sama dbałość o wizualną przejrzystość posłużyła jako wytyczna przy projektowaniu interfejsu serwisu internetowego, w którym kluczową rolę powierzyłem fotografii i materiałom wideo. Karta nieruchomości została zaplanowana tak, aby w naturalny sposób prowadzić użytkownika od narracyjnego opisu po lewej stronie do przejrzystego panelu ze specyfikacją techniczną po prawej. Chcąc dodatkowo podkreślić pozycję Epic jako eksperta rynkowego, zaprojektowałem i wdrożyłem autorski moduł Valor EPIC en la zona, który zestawiamy bezpośrednio cenę za metr kwadratowy danej nieruchomości ze średnią rynkową dla całej dzielnicy.</t>
+  </si>
+  <si>
+    <t>This focus on visual clarity guided the design of the website’s user interface, where high-resolution imagery and video walkthroughs take center stage. I structured the property listing pages to seamlessly guide users from rich editorial storytelling on the left to an organized technical spec panel on the right. To further reinforce Epic's standing as a trusted market authority, I introduced a custom Valor EPIC en la zona module, which directly benchmarks a property's price per square meter against the neighborhood average.</t>
+  </si>
+  <si>
+    <t>Esta misma búsqueda de claridad guió el diseño de la interfaz web, asignando el papel protagónico a la fotografía de alta calidad y a los recorridos en video. La ficha de propiedad se organizó de manera intuitiva para guiar al usuario desde la descripción narrativa a la izquierda hacia un panel funcional de especificaciones técnicas a la derecha. Con el fin de consolidar a Epic como una autoridad en el sector, integré el módulo exclusivo Valor EPIC en la zona, el cual contrasta directamente el precio por metro cuadrado de la propiedad con el promedio del vecindario.</t>
+  </si>
+  <si>
     <t>Sekcja 05</t>
   </si>
   <si>
     <t>sections.4.label</t>
   </si>
   <si>
+    <t>Architektura Strony &amp; Webflow</t>
+  </si>
+  <si>
+    <t>Platform Architecture</t>
+  </si>
+  <si>
+    <t>Arquitectura en Webflow CMS</t>
+  </si>
+  <si>
     <t>sections.4.title</t>
   </si>
   <si>
+    <t>Skalowalny system Webflow CMS i elastyczność edycji</t>
+  </si>
+  <si>
+    <t>Seamless Content Management Built for Growth</t>
+  </si>
+  <si>
+    <t>Estructura escalable y gestión de contenidos sin complicaciones</t>
+  </si>
+  <si>
     <t>sections.4.text</t>
   </si>
   <si>
+    <t>Przemyślana architektura interfejsu wymagała równie sprawnego zaplecza technologicznego, dlatego zdecydowaliśmy się na migrację serwisu z przestarzałego WordPressa na platformę Webflow. Na potrzeby projektu zbudowałem elastyczną strukturę CMS z osobnymi kolekcjami bazodanowymi dla nieruchomości oraz artykułów eksperckich. Dzięki temu założyciele agencji zyskali pełną swobodę w sprawnej publikacji i edycji ofert bez ryzyka naruszenia spójności visual designu. Tak przygotowany fundament otwiera również drogę do łatwej rozbudowy serwisu o zaawansowane filtrowanie oraz dedykowane strony docelowe dla poszczególnych dzielnic.</t>
+  </si>
+  <si>
+    <t>To support this thoughtful interface, we migrated the website from an outdated WordPress environment over to Webflow. I engineered a tailored CMS architecture featuring dedicated database collections for properties and market insights. This grants the founders complete autonomy to publish and edit listings smoothly without risking design integrity. Additionally, the underlying system was structured to scale effortlessly, allowing for future expansions like advanced multi-filtering and dedicated neighborhood landing pages.</t>
+  </si>
+  <si>
+    <t>Para respaldar esta experiencia de usuario, realizamos la transición del sitio desde WordPress hacia Webflow. Diseñé una arquitectura CMS a medida con colecciones independientes para propiedades y artículos de análisis. Gracias a esta estructura, los fundadores cuentan con total autonomía para publicar y modificar inmuebles de forma ágil sin alterar la armonía del diseño. Asimismo, la infraestructura quedó preparada para escalar fácilmente mediante la incorporación de filtros avanzados y páginas dedicadas a zonas específicas.</t>
+  </si>
+  <si>
     <t>Sekcja 06</t>
   </si>
   <si>
     <t>sections.5.label</t>
   </si>
   <si>
+    <t>Strategia Konwersji</t>
+  </si>
+  <si>
+    <t>Conversion Strategy</t>
+  </si>
+  <si>
+    <t>Estrategia de conversión</t>
+  </si>
+  <si>
     <t>sections.5.title</t>
   </si>
   <si>
+    <t>Prosty kontakt i przemyślana optymalizacja konwersji</t>
+  </si>
+  <si>
+    <t>Streamlined Inquiries &amp; Data-Driven Optimization</t>
+  </si>
+  <si>
+    <t>Contacto directo y optimización continua de conversión</t>
+  </si>
+  <si>
     <t>sections.5.text</t>
   </si>
   <si>
+    <t>Ostatnim elementem układanki było stworzenie beztarciowej ścieżki konwersji, która zamienia zainteresowanie ofertą w bezpośredni kontakt z agencją. Zaprojektowałem główny przycisk akcji tak, aby wywoływał formularz powiązany bezpośrednio z aktualnie przeglądaną nieruchomością. Uwzględniając specyfikę lokalnego rynku, gdzie WhatsApp jest głównym narzędziem biznesowym, wdrożyłem szybki kontakt w nawigacji głównej. Cała struktura serwisu powstała z myślą o stałej analityce, co umożliwia łatwe prowadzenie testów A/B i ciągłą optymalizację wyników.</t>
+  </si>
+  <si>
+    <t>The final piece of the strategy focused on building a frictionless conversion pathway that seamlessly turns casual browsing into active inquiries. I designed the main call-to-action to open a contextual contact modal linked directly to the specific property being viewed. Recognizing that WhatsApp serves as the primary communication hub in Panama, I integrated a direct chat trigger right into the main navigation. The entire page architecture was engineered to support ongoing analytics, paving the way for straightforward A/B testing and continuous conversion rate optimization.</t>
+  </si>
+  <si>
+    <t>El paso final de la estrategia consistió en crear un embudo de conversión sin fricciones que facilite el paso de la navegación a la consulta directa. El botón de acción principal despliega un formulario contextual vinculado automáticamente a la ficha del inmueble seleccionado. Entendiendo que WhatsApp es la herramienta de comunicación comercial por excelencia en Panamá, integré un acceso directo en el menú de navegación principal. Toda la estructura de la página se concibió para facilitar la medición constante, permitiendo realizar pruebas A/B y optimizar los resultados de forma continua.</t>
+  </si>
+  <si>
     <t>Sekcja 07</t>
   </si>
   <si>
@@ -495,47 +578,104 @@
     <t>sections.7.label</t>
   </si>
   <si>
-    <t>SUMMARY</t>
-  </si>
-  <si>
-    <t>PODSUMOWANIE</t>
-  </si>
-  <si>
-    <t>Resultado</t>
-  </si>
-  <si>
     <t>sections.7.title</t>
   </si>
   <si>
-    <t>Transforming a bootstrapped logo into a cohesive, scalable design system.</t>
-  </si>
-  <si>
-    <t>Transformacja budżetowego logo w spójny i gotowy do skalowania system wizualny.</t>
-  </si>
-  <si>
-    <t>De un logotipo básico a un sistema de marca sólido, coherente y listo para escalar.</t>
-  </si>
-  <si>
     <t>sections.7.text</t>
   </si>
   <si>
-    <t>The rebranding elevated Epic Realty's market perception, transforming a basic logo into a mature, premium brand identity. The synergy between the custom wordmark, the multi-faceted emblem, and the bold architectural typography gave the agency an instant, unmistakable presence in Panama.
-As part of the deliverable, I built a comprehensive social media template system (posts, stories, property listings), empowering their internal team to effortlessly create consistent, high-impact marketing assets. This design foundation also laid the groundwork for their upcoming custom website.</t>
-  </si>
-  <si>
-    <t>Przeprowadzony rebranding całkowicie zmienił percepcję Epic Realty, przekształcając budżetowy wizerunek w dojrzałą, unikalną markę z sektora premium. Połączenie autorskiej typografii znaku, przemyślanej symboliki sygnetu oraz odważnego kroju Barlow Condensed dało firmie natychmiastową rozpoznawalność na rynku panamskim.
-W ramach wdrożenia przygotowałem kompletny system szablonów dla mediów społecznościowych (posty, relacje, prezentacje ofert), który umożliwił zespołowi łatwe i powtarzalne budowanie spójnej komunikacji. Całość prac brandowych stała się bezpośrednim i solidnym fundamentem pod projekt nowej, dedykowanej strony internetowej.</t>
-  </si>
-  <si>
-    <t>El rebranding transformó por completo la percepción de Epic Realty, evolucionando una imagen inicial en una marca sofisticada y distintiva dentro del segmento de lujo. La sinergia entre el logotipo a medida, la riqueza simbólica del isotipo y el uso estratégico de Barlow Condensed le dio a la agencia una presencia memorable en Panamá.
-Como parte del proyecto, entregué un sistema integral de plantillas para redes sociales (publicaciones, historias y fichas de propiedades), permitiendo al equipo interno mantener una comunicación coherente de forma sencilla. Este trabajo de identidad sirvió además como la base gráfica para el desarrollo de su nuevo sitio web.</t>
+    <t>Sekcja 09</t>
+  </si>
+  <si>
+    <t>sections.8.label</t>
+  </si>
+  <si>
+    <t>sections.8.title</t>
+  </si>
+  <si>
+    <t>sections.8.text</t>
+  </si>
+  <si>
+    <t>Sekcja 10 (Summary)</t>
+  </si>
+  <si>
+    <t>sections.9.label</t>
+  </si>
+  <si>
+    <t>Podsumowanie</t>
+  </si>
+  <si>
+    <t>Summary</t>
+  </si>
+  <si>
+    <t>Resumen</t>
+  </si>
+  <si>
+    <t>Ostatnia sekcja: domyślnie Summary / Podsumowanie / Resumen. Zawsze białe tło.</t>
+  </si>
+  <si>
+    <t>sections.9.title</t>
+  </si>
+  <si>
+    <t>Nowy standard luksusu na panamskim rynku</t>
+  </si>
+  <si>
+    <t>A Solid Foundation for Panama's Premier Property Brand</t>
+  </si>
+  <si>
+    <t>Consolidando una nueva presencia en el mercado inmobiliario</t>
+  </si>
+  <si>
+    <t>sections.9.text</t>
+  </si>
+  <si>
+    <t>Projekt dla Epic Realty połączył wyrazistą tożsamość marki z wydajną platformą Webflow CMS. Odrzucenie szablonowych rozwiązań na rzecz unikalnej typografii Barlow Condensed, dopracowanej palety barw oraz przejrzystej architektury informacji pozwoliło zbudować wizerunek godny lidera rynku. Platforma stanowi elastyczny, przygotowany do dalszego rozwoju serwis, który pozwala marce wyznaczać nowe standardy w segmencie nieruchomości luksusowych.</t>
+  </si>
+  <si>
+    <t>The Epic Realty project successfully bridges high-end branding with modern web architecture. Replacing generic industry templates with Barlow Condensed typography, a sophisticated color strategy, and clear information hierarchy positions Epic to command market authority. The platform provides a scalable foundation that empowers the brand to set new standards in luxury real estate.</t>
+  </si>
+  <si>
+    <t>El proyecto de Epic Realty une una identidad visual sofisticada con la flexibilidad de Webflow CMS. Al reemplazar los esquemas convencionales por la tipografía Barlow Condensed, una paleta de colores elegante y una estructura de información clara, la marca queda posicionada para liderar su segmento. La plataforma constituye una base sólida y escalable que permite a la empresa establecer nuevos estándares en el sector de lujo.</t>
+  </si>
+  <si>
+    <t>Opinia klienta</t>
+  </si>
+  <si>
+    <t>quoteLabel</t>
+  </si>
+  <si>
+    <t>Client review</t>
+  </si>
+  <si>
+    <t>Opinión del cliente</t>
+  </si>
+  <si>
+    <t>Etykieta nad cytatem, bez [ ]. Puste = domyślne [Client review] / [Opinia klienta] / [Opinión del cliente].</t>
+  </si>
+  <si>
+    <t>quote</t>
+  </si>
+  <si>
+    <t>Treść cytatu / opinii klienta. Umieszczana pod sekcją Summary. Puste = sekcja ukryta.</t>
+  </si>
+  <si>
+    <t>quoteAuthor</t>
+  </si>
+  <si>
+    <t>Imię i nazwisko autora cytatu (np. Nedelka Velasco).</t>
+  </si>
+  <si>
+    <t>quoteRole</t>
+  </si>
+  <si>
+    <t>Stanowisko / firma autora cytatu (np. CEO of NRV).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -545,7 +685,7 @@
     <font>
       <b/>
       <sz val="16.0"/>
-      <color theme="1"/>
+      <color rgb="FF111111"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -556,9 +696,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12.0"/>
-      <color theme="1"/>
+      <i/>
+      <sz val="10.0"/>
+      <color rgb="FF666666"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -567,8 +707,15 @@
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12.0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -595,53 +742,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF7F7F7"/>
+        <bgColor rgb="FFF7F7F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE599"/>
-        <bgColor rgb="FFFFE599"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF3F3F3"/>
-        <bgColor rgb="FFF3F3F3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF7F7F7"/>
-        <bgColor rgb="FFF7F7F7"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border/>
     <border>
       <left/>
-      <right/>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
       <right/>
       <top/>
       <bottom/>
@@ -650,76 +765,38 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="13">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="8" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="8" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="8" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="8" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -947,7 +1024,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="100.0"/>
+    <col customWidth="1" min="1" max="1" width="110.0"/>
     <col customWidth="1" min="2" max="26" width="8.71"/>
   </cols>
   <sheetData>
@@ -955,95 +1032,95 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
-      <c r="V1" s="2"/>
-      <c r="W1" s="2"/>
-      <c r="X1" s="2"/>
-      <c r="Y1" s="2"/>
-      <c r="Z1" s="2"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="4"/>
-      <c r="Y3" s="4"/>
-      <c r="Z3" s="4"/>
-    </row>
-    <row r="4" ht="39.75" customHeight="1">
-      <c r="A4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="5"/>
-      <c r="T4" s="5"/>
-      <c r="U4" s="5"/>
-      <c r="V4" s="5"/>
-      <c r="W4" s="5"/>
-      <c r="X4" s="5"/>
-      <c r="Y4" s="5"/>
-      <c r="Z4" s="5"/>
-    </row>
-    <row r="5" ht="39.75" customHeight="1">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
+      <c r="V2" s="3"/>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+      <c r="Y2" s="3"/>
+      <c r="Z2" s="3"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
+      <c r="X4" s="6"/>
+      <c r="Y4" s="6"/>
+      <c r="Z4" s="6"/>
+    </row>
+    <row r="5" ht="25.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -1071,9 +1148,9 @@
       <c r="Y5" s="5"/>
       <c r="Z5" s="5"/>
     </row>
-    <row r="6" ht="39.75" customHeight="1">
+    <row r="6" ht="25.5" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -1101,9 +1178,9 @@
       <c r="Y6" s="5"/>
       <c r="Z6" s="5"/>
     </row>
-    <row r="7" ht="39.75" customHeight="1">
+    <row r="7" ht="25.5" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -1131,99 +1208,99 @@
       <c r="Y7" s="5"/>
       <c r="Z7" s="5"/>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="4"/>
-      <c r="R9" s="4"/>
-      <c r="S9" s="4"/>
-      <c r="T9" s="4"/>
-      <c r="U9" s="4"/>
-      <c r="V9" s="4"/>
-      <c r="W9" s="4"/>
-      <c r="X9" s="4"/>
-      <c r="Y9" s="4"/>
-      <c r="Z9" s="4"/>
-    </row>
-    <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
-      <c r="P10" s="5"/>
-      <c r="Q10" s="5"/>
-      <c r="R10" s="5"/>
-      <c r="S10" s="5"/>
-      <c r="T10" s="5"/>
-      <c r="U10" s="5"/>
-      <c r="V10" s="5"/>
-      <c r="W10" s="5"/>
-      <c r="X10" s="5"/>
-      <c r="Y10" s="5"/>
-      <c r="Z10" s="5"/>
-    </row>
-    <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="5"/>
-      <c r="R11" s="5"/>
-      <c r="S11" s="5"/>
-      <c r="T11" s="5"/>
-      <c r="U11" s="5"/>
-      <c r="V11" s="5"/>
-      <c r="W11" s="5"/>
-      <c r="X11" s="5"/>
-      <c r="Y11" s="5"/>
-      <c r="Z11" s="5"/>
-    </row>
-    <row r="12" ht="39.75" customHeight="1">
+    <row r="8" ht="25.5" customHeight="1">
+      <c r="A8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="5"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="5"/>
+      <c r="W8" s="5"/>
+      <c r="X8" s="5"/>
+      <c r="Y8" s="5"/>
+      <c r="Z8" s="5"/>
+    </row>
+    <row r="9" ht="25.5" customHeight="1">
+      <c r="A9" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="5"/>
+      <c r="X9" s="5"/>
+      <c r="Y9" s="5"/>
+      <c r="Z9" s="5"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="6"/>
+      <c r="S11" s="6"/>
+      <c r="T11" s="6"/>
+      <c r="U11" s="6"/>
+      <c r="V11" s="6"/>
+      <c r="W11" s="6"/>
+      <c r="X11" s="6"/>
+      <c r="Y11" s="6"/>
+      <c r="Z11" s="6"/>
+    </row>
+    <row r="12" ht="25.5" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1251,65 +1328,65 @@
       <c r="Y12" s="5"/>
       <c r="Z12" s="5"/>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="4"/>
-      <c r="R14" s="4"/>
-      <c r="S14" s="4"/>
-      <c r="T14" s="4"/>
-      <c r="U14" s="4"/>
-      <c r="V14" s="4"/>
-      <c r="W14" s="4"/>
-      <c r="X14" s="4"/>
-      <c r="Y14" s="4"/>
-      <c r="Z14" s="4"/>
-    </row>
-    <row r="15" ht="39.75" customHeight="1">
-      <c r="A15" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="5"/>
-      <c r="P15" s="5"/>
-      <c r="Q15" s="5"/>
-      <c r="R15" s="5"/>
-      <c r="S15" s="5"/>
-      <c r="T15" s="5"/>
-      <c r="U15" s="5"/>
-      <c r="V15" s="5"/>
-      <c r="W15" s="5"/>
-      <c r="X15" s="5"/>
-      <c r="Y15" s="5"/>
-      <c r="Z15" s="5"/>
+    <row r="13" ht="25.5" customHeight="1">
+      <c r="A13" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5"/>
+      <c r="S13" s="5"/>
+      <c r="T13" s="5"/>
+      <c r="U13" s="5"/>
+      <c r="V13" s="5"/>
+      <c r="W13" s="5"/>
+      <c r="X13" s="5"/>
+      <c r="Y13" s="5"/>
+      <c r="Z13" s="5"/>
+    </row>
+    <row r="14" ht="25.5" customHeight="1">
+      <c r="A14" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+      <c r="R14" s="5"/>
+      <c r="S14" s="5"/>
+      <c r="T14" s="5"/>
+      <c r="U14" s="5"/>
+      <c r="V14" s="5"/>
+      <c r="W14" s="5"/>
+      <c r="X14" s="5"/>
+      <c r="Y14" s="5"/>
+      <c r="Z14" s="5"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -2306,67 +2383,71 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="14.0"/>
+    <col customWidth="1" min="1" max="1" width="24.0"/>
     <col customWidth="1" min="2" max="2" width="22.0"/>
-    <col customWidth="1" min="3" max="5" width="56.0"/>
-    <col customWidth="1" min="6" max="6" width="52.0"/>
+    <col customWidth="1" min="3" max="5" width="50.0"/>
+    <col customWidth="1" min="6" max="6" width="54.0"/>
     <col customWidth="1" min="7" max="26" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="3"/>
-      <c r="X1" s="3"/>
-      <c r="Y1" s="3"/>
-      <c r="Z1" s="3"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+      <c r="Z1" s="2"/>
     </row>
     <row r="2" ht="31.5" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="D2" s="8"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
@@ -2390,23 +2471,23 @@
       <c r="Z2" s="5"/>
     </row>
     <row r="3" ht="31.5" customHeight="1">
-      <c r="A3" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>34</v>
+      <c r="A3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
@@ -2430,23 +2511,23 @@
       <c r="Z3" s="5"/>
     </row>
     <row r="4" ht="31.5" customHeight="1">
-      <c r="A4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>40</v>
+      <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
@@ -2470,23 +2551,23 @@
       <c r="Z4" s="5"/>
     </row>
     <row r="5" ht="31.5" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="16" t="b">
-        <v>0</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>42</v>
+      <c r="A5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>32</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
@@ -2510,23 +2591,23 @@
       <c r="Z5" s="5"/>
     </row>
     <row r="6" ht="31.5" customHeight="1">
-      <c r="A6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>44</v>
+      <c r="A6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>45</v>
+        <v>37</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
@@ -2549,24 +2630,24 @@
       <c r="Y6" s="5"/>
       <c r="Z6" s="5"/>
     </row>
-    <row r="7" ht="24.0" customHeight="1">
-      <c r="A7" s="6" t="s">
+    <row r="7" ht="25.5" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="E7" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>51</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
@@ -2590,23 +2671,23 @@
       <c r="Z7" s="5"/>
     </row>
     <row r="8" ht="31.5" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>53</v>
+      <c r="A8" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>37</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>54</v>
+        <v>37</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>49</v>
       </c>
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
@@ -2629,24 +2710,24 @@
       <c r="Y8" s="5"/>
       <c r="Z8" s="5"/>
     </row>
-    <row r="9" ht="24.0" customHeight="1">
-      <c r="A9" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="D9" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>57</v>
+    <row r="9" ht="25.5" customHeight="1">
+      <c r="A9" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>53</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
@@ -2670,23 +2751,23 @@
       <c r="Z9" s="5"/>
     </row>
     <row r="10" ht="31.5" customHeight="1">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="D10" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
@@ -2709,24 +2790,24 @@
       <c r="Y10" s="5"/>
       <c r="Z10" s="5"/>
     </row>
-    <row r="11" ht="31.5" customHeight="1">
-      <c r="A11" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="6" t="s">
+    <row r="11" ht="25.5" customHeight="1">
+      <c r="A11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>67</v>
       </c>
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
@@ -2749,24 +2830,24 @@
       <c r="Y11" s="5"/>
       <c r="Z11" s="5"/>
     </row>
-    <row r="12" ht="24.0" customHeight="1">
-      <c r="A12" s="6" t="s">
+    <row r="12" ht="25.5" customHeight="1">
+      <c r="A12" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="F12" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>73</v>
       </c>
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
@@ -2789,24 +2870,24 @@
       <c r="Y12" s="5"/>
       <c r="Z12" s="5"/>
     </row>
-    <row r="13" ht="24.0" customHeight="1">
-      <c r="A13" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="D13" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="E13" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="F13" s="6" t="s">
+    <row r="13" ht="25.5" customHeight="1">
+      <c r="A13" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>73</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>69</v>
       </c>
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
@@ -2829,24 +2910,24 @@
       <c r="Y13" s="5"/>
       <c r="Z13" s="5"/>
     </row>
-    <row r="14" ht="24.0" customHeight="1">
-      <c r="A14" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>79</v>
+    <row r="14" ht="25.5" customHeight="1">
+      <c r="A14" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>75</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>69</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
@@ -2869,24 +2950,24 @@
       <c r="Y14" s="5"/>
       <c r="Z14" s="5"/>
     </row>
-    <row r="15" ht="24.0" customHeight="1">
-      <c r="A15" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="D15" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="E15" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>73</v>
+    <row r="15" ht="25.5" customHeight="1">
+      <c r="A15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>69</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
@@ -2909,24 +2990,24 @@
       <c r="Y15" s="5"/>
       <c r="Z15" s="5"/>
     </row>
-    <row r="16" ht="24.0" customHeight="1">
-      <c r="A16" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="C16" s="7">
-        <v>2025.0</v>
-      </c>
-      <c r="D16" s="19">
-        <v>2025.0</v>
-      </c>
-      <c r="E16" s="20">
-        <v>2025.0</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>84</v>
+    <row r="16" ht="25.5" customHeight="1">
+      <c r="A16" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>81</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
@@ -2949,24 +3030,24 @@
       <c r="Y16" s="5"/>
       <c r="Z16" s="5"/>
     </row>
-    <row r="17" ht="24.0" customHeight="1">
-      <c r="A17" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>86</v>
+    <row r="17" ht="25.5" customHeight="1">
+      <c r="A17" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>83</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E17" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>87</v>
+        <v>14</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>84</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="5"/>
@@ -2989,24 +3070,24 @@
       <c r="Y17" s="5"/>
       <c r="Z17" s="5"/>
     </row>
-    <row r="18" ht="24.0" customHeight="1">
-      <c r="A18" s="6" t="s">
+    <row r="18" ht="25.5" customHeight="1">
+      <c r="A18" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="E18" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>89</v>
+      <c r="C18" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>86</v>
       </c>
       <c r="G18" s="5"/>
       <c r="H18" s="5"/>
@@ -3030,23 +3111,23 @@
       <c r="Z18" s="5"/>
     </row>
     <row r="19" ht="31.5" customHeight="1">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="F19" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="G19" s="5"/>
       <c r="H19" s="5"/>
@@ -3069,24 +3150,24 @@
       <c r="Y19" s="5"/>
       <c r="Z19" s="5"/>
     </row>
-    <row r="20" ht="24.0" customHeight="1">
-      <c r="A20" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B20" s="6" t="s">
+    <row r="20" ht="25.5" customHeight="1">
+      <c r="A20" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>95</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>99</v>
       </c>
       <c r="G20" s="5"/>
       <c r="H20" s="5"/>
@@ -3109,24 +3190,24 @@
       <c r="Y20" s="5"/>
       <c r="Z20" s="5"/>
     </row>
-    <row r="21" ht="24.0" customHeight="1">
-      <c r="A21" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B21" s="6" t="s">
+    <row r="21" ht="162.75" customHeight="1">
+      <c r="A21" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>100</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="D21" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>103</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>104</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="5"/>
@@ -3150,23 +3231,23 @@
       <c r="Z21" s="5"/>
     </row>
     <row r="22" ht="31.5" customHeight="1">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
@@ -3189,24 +3270,24 @@
       <c r="Y22" s="5"/>
       <c r="Z22" s="5"/>
     </row>
-    <row r="23" ht="24.0" customHeight="1">
-      <c r="A23" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C23" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="D23" s="17" t="s">
-        <v>113</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>115</v>
+    <row r="23" ht="25.5" customHeight="1">
+      <c r="A23" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="5"/>
@@ -3229,24 +3310,24 @@
       <c r="Y23" s="5"/>
       <c r="Z23" s="5"/>
     </row>
-    <row r="24" ht="31.5" customHeight="1">
-      <c r="A24" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>117</v>
+    <row r="24" ht="165.0" customHeight="1">
+      <c r="A24" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>112</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>120</v>
+        <v>113</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="5"/>
@@ -3270,23 +3351,23 @@
       <c r="Z24" s="5"/>
     </row>
     <row r="25" ht="31.5" customHeight="1">
-      <c r="A25" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="C25" s="16" t="s">
-        <v>123</v>
-      </c>
-      <c r="D25" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="E25" s="18" t="s">
-        <v>125</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>110</v>
+      <c r="A25" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="G25" s="5"/>
       <c r="H25" s="5"/>
@@ -3309,24 +3390,24 @@
       <c r="Y25" s="5"/>
       <c r="Z25" s="5"/>
     </row>
-    <row r="26" ht="24.0" customHeight="1">
-      <c r="A26" s="6" t="s">
+    <row r="26" ht="25.5" customHeight="1">
+      <c r="A26" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>127</v>
+      <c r="C26" s="11" t="s">
+        <v>122</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>115</v>
+        <v>123</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="G26" s="5"/>
       <c r="H26" s="5"/>
@@ -3349,24 +3430,24 @@
       <c r="Y26" s="5"/>
       <c r="Z26" s="5"/>
     </row>
-    <row r="27" ht="31.5" customHeight="1">
-      <c r="A27" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C27" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="D27" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="E27" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>120</v>
+    <row r="27" ht="119.25" customHeight="1">
+      <c r="A27" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="G27" s="5"/>
       <c r="H27" s="5"/>
@@ -3390,23 +3471,23 @@
       <c r="Z27" s="5"/>
     </row>
     <row r="28" ht="31.5" customHeight="1">
-      <c r="A28" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D28" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>110</v>
+      <c r="A28" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="E28" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="G28" s="5"/>
       <c r="H28" s="5"/>
@@ -3429,24 +3510,24 @@
       <c r="Y28" s="5"/>
       <c r="Z28" s="5"/>
     </row>
-    <row r="29" ht="24.0" customHeight="1">
-      <c r="A29" s="6" t="s">
+    <row r="29" ht="25.5" customHeight="1">
+      <c r="A29" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="C29" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="C29" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E29" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>115</v>
+      <c r="E29" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="G29" s="5"/>
       <c r="H29" s="5"/>
@@ -3469,24 +3550,24 @@
       <c r="Y29" s="5"/>
       <c r="Z29" s="5"/>
     </row>
-    <row r="30" ht="31.5" customHeight="1">
-      <c r="A30" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E30" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>120</v>
+    <row r="30" ht="109.5" customHeight="1">
+      <c r="A30" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="G30" s="5"/>
       <c r="H30" s="5"/>
@@ -3510,23 +3591,23 @@
       <c r="Z30" s="5"/>
     </row>
     <row r="31" ht="31.5" customHeight="1">
-      <c r="A31" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D31" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E31" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>110</v>
+      <c r="A31" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="G31" s="5"/>
       <c r="H31" s="5"/>
@@ -3549,24 +3630,24 @@
       <c r="Y31" s="5"/>
       <c r="Z31" s="5"/>
     </row>
-    <row r="32" ht="24.0" customHeight="1">
-      <c r="A32" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D32" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E32" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>115</v>
+    <row r="32" ht="25.5" customHeight="1">
+      <c r="A32" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="G32" s="5"/>
       <c r="H32" s="5"/>
@@ -3589,24 +3670,24 @@
       <c r="Y32" s="5"/>
       <c r="Z32" s="5"/>
     </row>
-    <row r="33" ht="31.5" customHeight="1">
-      <c r="A33" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="C33" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D33" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E33" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>120</v>
+    <row r="33" ht="145.5" customHeight="1">
+      <c r="A33" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="G33" s="5"/>
       <c r="H33" s="5"/>
@@ -3630,23 +3711,23 @@
       <c r="Z33" s="5"/>
     </row>
     <row r="34" ht="31.5" customHeight="1">
-      <c r="A34" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D34" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E34" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>110</v>
+      <c r="A34" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="G34" s="5"/>
       <c r="H34" s="5"/>
@@ -3669,24 +3750,24 @@
       <c r="Y34" s="5"/>
       <c r="Z34" s="5"/>
     </row>
-    <row r="35" ht="24.0" customHeight="1">
-      <c r="A35" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="C35" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D35" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E35" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>115</v>
+    <row r="35" ht="25.5" customHeight="1">
+      <c r="A35" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="G35" s="5"/>
       <c r="H35" s="5"/>
@@ -3709,24 +3790,24 @@
       <c r="Y35" s="5"/>
       <c r="Z35" s="5"/>
     </row>
-    <row r="36" ht="31.5" customHeight="1">
-      <c r="A36" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D36" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E36" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>120</v>
+    <row r="36" ht="145.5" customHeight="1">
+      <c r="A36" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="E36" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
@@ -3750,23 +3831,23 @@
       <c r="Z36" s="5"/>
     </row>
     <row r="37" ht="31.5" customHeight="1">
-      <c r="A37" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="C37" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D37" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E37" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>110</v>
+      <c r="A37" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="G37" s="5"/>
       <c r="H37" s="5"/>
@@ -3789,24 +3870,24 @@
       <c r="Y37" s="5"/>
       <c r="Z37" s="5"/>
     </row>
-    <row r="38" ht="24.0" customHeight="1">
-      <c r="A38" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="C38" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D38" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E38" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F38" s="6" t="s">
-        <v>115</v>
+    <row r="38" ht="25.5" customHeight="1">
+      <c r="A38" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C38" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="E38" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="G38" s="5"/>
       <c r="H38" s="5"/>
@@ -3829,24 +3910,24 @@
       <c r="Y38" s="5"/>
       <c r="Z38" s="5"/>
     </row>
-    <row r="39" ht="31.5" customHeight="1">
-      <c r="A39" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="C39" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D39" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E39" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>120</v>
+    <row r="39" ht="138.0" customHeight="1">
+      <c r="A39" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="G39" s="5"/>
       <c r="H39" s="5"/>
@@ -3870,23 +3951,23 @@
       <c r="Z39" s="5"/>
     </row>
     <row r="40" ht="31.5" customHeight="1">
-      <c r="A40" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D40" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E40" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>110</v>
+      <c r="A40" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E40" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="G40" s="5"/>
       <c r="H40" s="5"/>
@@ -3909,24 +3990,24 @@
       <c r="Y40" s="5"/>
       <c r="Z40" s="5"/>
     </row>
-    <row r="41" ht="24.0" customHeight="1">
-      <c r="A41" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>152</v>
+    <row r="41" ht="25.5" customHeight="1">
+      <c r="A41" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>183</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D41" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E41" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>115</v>
+        <v>14</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
@@ -3950,23 +4031,23 @@
       <c r="Z41" s="5"/>
     </row>
     <row r="42" ht="31.5" customHeight="1">
-      <c r="A42" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D42" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E42" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>120</v>
+      <c r="A42" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="G42" s="5"/>
       <c r="H42" s="5"/>
@@ -3990,23 +4071,23 @@
       <c r="Z42" s="5"/>
     </row>
     <row r="43" ht="31.5" customHeight="1">
-      <c r="A43" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="C43" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="D43" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="E43" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>110</v>
+      <c r="A43" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="G43" s="5"/>
       <c r="H43" s="5"/>
@@ -4029,24 +4110,24 @@
       <c r="Y43" s="5"/>
       <c r="Z43" s="5"/>
     </row>
-    <row r="44" ht="24.0" customHeight="1">
-      <c r="A44" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="C44" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="D44" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="E44" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>115</v>
+    <row r="44" ht="25.5" customHeight="1">
+      <c r="A44" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="G44" s="5"/>
       <c r="H44" s="5"/>
@@ -4070,23 +4151,23 @@
       <c r="Z44" s="5"/>
     </row>
     <row r="45" ht="31.5" customHeight="1">
-      <c r="A45" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>164</v>
-      </c>
-      <c r="D45" s="17" t="s">
-        <v>165</v>
-      </c>
-      <c r="E45" s="18" t="s">
-        <v>166</v>
-      </c>
-      <c r="F45" s="6" t="s">
-        <v>120</v>
+      <c r="A45" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="G45" s="5"/>
       <c r="H45" s="5"/>
@@ -4109,16 +4190,406 @@
       <c r="Y45" s="5"/>
       <c r="Z45" s="5"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1"/>
-    <row r="47" ht="15.75" customHeight="1"/>
-    <row r="48" ht="15.75" customHeight="1"/>
-    <row r="49" ht="15.75" customHeight="1"/>
-    <row r="50" ht="15.75" customHeight="1"/>
-    <row r="51" ht="15.75" customHeight="1"/>
-    <row r="52" ht="15.75" customHeight="1"/>
-    <row r="53" ht="15.75" customHeight="1"/>
-    <row r="54" ht="15.75" customHeight="1"/>
-    <row r="55" ht="15.75" customHeight="1"/>
+    <row r="46" ht="31.5" customHeight="1">
+      <c r="A46" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E46" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G46" s="5"/>
+      <c r="H46" s="5"/>
+      <c r="I46" s="5"/>
+      <c r="J46" s="5"/>
+      <c r="K46" s="5"/>
+      <c r="L46" s="5"/>
+      <c r="M46" s="5"/>
+      <c r="N46" s="5"/>
+      <c r="O46" s="5"/>
+      <c r="P46" s="5"/>
+      <c r="Q46" s="5"/>
+      <c r="R46" s="5"/>
+      <c r="S46" s="5"/>
+      <c r="T46" s="5"/>
+      <c r="U46" s="5"/>
+      <c r="V46" s="5"/>
+      <c r="W46" s="5"/>
+      <c r="X46" s="5"/>
+      <c r="Y46" s="5"/>
+      <c r="Z46" s="5"/>
+    </row>
+    <row r="47" ht="25.5" customHeight="1">
+      <c r="A47" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E47" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5"/>
+      <c r="I47" s="5"/>
+      <c r="J47" s="5"/>
+      <c r="K47" s="5"/>
+      <c r="L47" s="5"/>
+      <c r="M47" s="5"/>
+      <c r="N47" s="5"/>
+      <c r="O47" s="5"/>
+      <c r="P47" s="5"/>
+      <c r="Q47" s="5"/>
+      <c r="R47" s="5"/>
+      <c r="S47" s="5"/>
+      <c r="T47" s="5"/>
+      <c r="U47" s="5"/>
+      <c r="V47" s="5"/>
+      <c r="W47" s="5"/>
+      <c r="X47" s="5"/>
+      <c r="Y47" s="5"/>
+      <c r="Z47" s="5"/>
+    </row>
+    <row r="48" ht="31.5" customHeight="1">
+      <c r="A48" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="K48" s="5"/>
+      <c r="L48" s="5"/>
+      <c r="M48" s="5"/>
+      <c r="N48" s="5"/>
+      <c r="O48" s="5"/>
+      <c r="P48" s="5"/>
+      <c r="Q48" s="5"/>
+      <c r="R48" s="5"/>
+      <c r="S48" s="5"/>
+      <c r="T48" s="5"/>
+      <c r="U48" s="5"/>
+      <c r="V48" s="5"/>
+      <c r="W48" s="5"/>
+      <c r="X48" s="5"/>
+      <c r="Y48" s="5"/>
+      <c r="Z48" s="5"/>
+    </row>
+    <row r="49" ht="31.5" customHeight="1">
+      <c r="A49" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="K49" s="5"/>
+      <c r="L49" s="5"/>
+      <c r="M49" s="5"/>
+      <c r="N49" s="5"/>
+      <c r="O49" s="5"/>
+      <c r="P49" s="5"/>
+      <c r="Q49" s="5"/>
+      <c r="R49" s="5"/>
+      <c r="S49" s="5"/>
+      <c r="T49" s="5"/>
+      <c r="U49" s="5"/>
+      <c r="V49" s="5"/>
+      <c r="W49" s="5"/>
+      <c r="X49" s="5"/>
+      <c r="Y49" s="5"/>
+      <c r="Z49" s="5"/>
+    </row>
+    <row r="50" ht="25.5" customHeight="1">
+      <c r="A50" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="E50" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+      <c r="I50" s="5"/>
+      <c r="J50" s="5"/>
+      <c r="K50" s="5"/>
+      <c r="L50" s="5"/>
+      <c r="M50" s="5"/>
+      <c r="N50" s="5"/>
+      <c r="O50" s="5"/>
+      <c r="P50" s="5"/>
+      <c r="Q50" s="5"/>
+      <c r="R50" s="5"/>
+      <c r="S50" s="5"/>
+      <c r="T50" s="5"/>
+      <c r="U50" s="5"/>
+      <c r="V50" s="5"/>
+      <c r="W50" s="5"/>
+      <c r="X50" s="5"/>
+      <c r="Y50" s="5"/>
+      <c r="Z50" s="5"/>
+    </row>
+    <row r="51" ht="96.0" customHeight="1">
+      <c r="A51" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="D51" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+      <c r="L51" s="5"/>
+      <c r="M51" s="5"/>
+      <c r="N51" s="5"/>
+      <c r="O51" s="5"/>
+      <c r="P51" s="5"/>
+      <c r="Q51" s="5"/>
+      <c r="R51" s="5"/>
+      <c r="S51" s="5"/>
+      <c r="T51" s="5"/>
+      <c r="U51" s="5"/>
+      <c r="V51" s="5"/>
+      <c r="W51" s="5"/>
+      <c r="X51" s="5"/>
+      <c r="Y51" s="5"/>
+      <c r="Z51" s="5"/>
+    </row>
+    <row r="52" ht="31.5" customHeight="1">
+      <c r="A52" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C52" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="E52" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="K52" s="5"/>
+      <c r="L52" s="5"/>
+      <c r="M52" s="5"/>
+      <c r="N52" s="5"/>
+      <c r="O52" s="5"/>
+      <c r="P52" s="5"/>
+      <c r="Q52" s="5"/>
+      <c r="R52" s="5"/>
+      <c r="S52" s="5"/>
+      <c r="T52" s="5"/>
+      <c r="U52" s="5"/>
+      <c r="V52" s="5"/>
+      <c r="W52" s="5"/>
+      <c r="X52" s="5"/>
+      <c r="Y52" s="5"/>
+      <c r="Z52" s="5"/>
+    </row>
+    <row r="53" ht="31.5" customHeight="1">
+      <c r="A53" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="G53" s="5"/>
+      <c r="H53" s="5"/>
+      <c r="I53" s="5"/>
+      <c r="J53" s="5"/>
+      <c r="K53" s="5"/>
+      <c r="L53" s="5"/>
+      <c r="M53" s="5"/>
+      <c r="N53" s="5"/>
+      <c r="O53" s="5"/>
+      <c r="P53" s="5"/>
+      <c r="Q53" s="5"/>
+      <c r="R53" s="5"/>
+      <c r="S53" s="5"/>
+      <c r="T53" s="5"/>
+      <c r="U53" s="5"/>
+      <c r="V53" s="5"/>
+      <c r="W53" s="5"/>
+      <c r="X53" s="5"/>
+      <c r="Y53" s="5"/>
+      <c r="Z53" s="5"/>
+    </row>
+    <row r="54" ht="25.5" customHeight="1">
+      <c r="A54" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E54" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="5"/>
+      <c r="K54" s="5"/>
+      <c r="L54" s="5"/>
+      <c r="M54" s="5"/>
+      <c r="N54" s="5"/>
+      <c r="O54" s="5"/>
+      <c r="P54" s="5"/>
+      <c r="Q54" s="5"/>
+      <c r="R54" s="5"/>
+      <c r="S54" s="5"/>
+      <c r="T54" s="5"/>
+      <c r="U54" s="5"/>
+      <c r="V54" s="5"/>
+      <c r="W54" s="5"/>
+      <c r="X54" s="5"/>
+      <c r="Y54" s="5"/>
+      <c r="Z54" s="5"/>
+    </row>
+    <row r="55" ht="25.5" customHeight="1">
+      <c r="A55" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C55" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="5"/>
+      <c r="K55" s="5"/>
+      <c r="L55" s="5"/>
+      <c r="M55" s="5"/>
+      <c r="N55" s="5"/>
+      <c r="O55" s="5"/>
+      <c r="P55" s="5"/>
+      <c r="Q55" s="5"/>
+      <c r="R55" s="5"/>
+      <c r="S55" s="5"/>
+      <c r="T55" s="5"/>
+      <c r="U55" s="5"/>
+      <c r="V55" s="5"/>
+      <c r="W55" s="5"/>
+      <c r="X55" s="5"/>
+      <c r="Y55" s="5"/>
+      <c r="Z55" s="5"/>
+    </row>
     <row r="56" ht="15.75" customHeight="1"/>
     <row r="57" ht="15.75" customHeight="1"/>
     <row r="58" ht="15.75" customHeight="1"/>
@@ -5065,7 +5536,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$1:$F$45"/>
+  <autoFilter ref="$A$1:$F$55"/>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="portrait"/>
@@ -5086,43 +5557,43 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="3"/>
-      <c r="X1" s="3"/>
-      <c r="Y1" s="3"/>
-      <c r="Z1" s="3"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+      <c r="Z1" s="2"/>
     </row>
     <row r="2" ht="27.75" customHeight="1">
       <c r="A2" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -5183,10 +5654,10 @@
     </row>
     <row r="4" ht="27.75" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -5215,10 +5686,10 @@
     </row>
     <row r="5" ht="27.75" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -5247,10 +5718,10 @@
     </row>
     <row r="6" ht="27.75" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -5279,10 +5750,10 @@
     </row>
     <row r="7" ht="27.75" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>

</xml_diff>